<commit_message>
data: Metas.xlsx atualizada com valores do Suas Vendas (2.667.169/mes = 32M anual)
</commit_message>
<xml_diff>
--- a/planilhas-snapshot/Metas.xlsx
+++ b/planilhas-snapshot/Metas.xlsx
@@ -463,7 +463,7 @@
         <v>2026</v>
       </c>
       <c r="C2" t="n">
-        <v>1100000</v>
+        <v>2667169</v>
       </c>
     </row>
     <row r="3">
@@ -476,7 +476,7 @@
         <v>2026</v>
       </c>
       <c r="C3" t="n">
-        <v>1100000</v>
+        <v>2667169</v>
       </c>
     </row>
     <row r="4">
@@ -489,7 +489,7 @@
         <v>2026</v>
       </c>
       <c r="C4" t="n">
-        <v>1100000</v>
+        <v>2667169</v>
       </c>
     </row>
     <row r="5">
@@ -502,7 +502,7 @@
         <v>2026</v>
       </c>
       <c r="C5" t="n">
-        <v>1100000</v>
+        <v>2667169</v>
       </c>
     </row>
     <row r="6">
@@ -515,7 +515,7 @@
         <v>2026</v>
       </c>
       <c r="C6" t="n">
-        <v>1100000</v>
+        <v>2667169</v>
       </c>
     </row>
     <row r="7">
@@ -528,7 +528,7 @@
         <v>2026</v>
       </c>
       <c r="C7" t="n">
-        <v>1100000</v>
+        <v>2667169</v>
       </c>
     </row>
     <row r="8">
@@ -541,7 +541,7 @@
         <v>2026</v>
       </c>
       <c r="C8" t="n">
-        <v>1100000</v>
+        <v>2667169</v>
       </c>
     </row>
     <row r="9">
@@ -554,7 +554,7 @@
         <v>2026</v>
       </c>
       <c r="C9" t="n">
-        <v>1100000</v>
+        <v>2667169</v>
       </c>
     </row>
     <row r="10">
@@ -567,7 +567,7 @@
         <v>2026</v>
       </c>
       <c r="C10" t="n">
-        <v>1100000</v>
+        <v>2667169</v>
       </c>
     </row>
     <row r="11">
@@ -580,7 +580,7 @@
         <v>2026</v>
       </c>
       <c r="C11" t="n">
-        <v>1100000</v>
+        <v>2667169</v>
       </c>
     </row>
     <row r="12">
@@ -593,7 +593,7 @@
         <v>2026</v>
       </c>
       <c r="C12" t="n">
-        <v>1100000</v>
+        <v>2667169</v>
       </c>
     </row>
     <row r="13">
@@ -606,7 +606,7 @@
         <v>2026</v>
       </c>
       <c r="C13" t="n">
-        <v>1100000</v>
+        <v>2667169</v>
       </c>
     </row>
   </sheetData>
@@ -3699,9 +3699,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -3709,9 +3707,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -3733,9 +3729,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -3764,9 +3758,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>

</xml_diff>